<commit_message>
hannah data table change
</commit_message>
<xml_diff>
--- a/data/2023_HRSWURN_Tables.xlsx
+++ b/data/2023_HRSWURN_Tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ARSMNSPP4DFG174\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\donoh132\Box\IWG_Breeding\Git_demo\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B57E4D5B-FAEA-4C0F-9AEA-2ABB4A1B0A5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8A7A450-8FC9-4E64-A2ED-8ED490FCBBE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="838" firstSheet="15" activeTab="26" xr2:uid="{BC65913E-1809-4B59-BE8F-B0869AF7DC59}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="838" firstSheet="18" activeTab="27" xr2:uid="{BC65913E-1809-4B59-BE8F-B0869AF7DC59}"/>
   </bookViews>
   <sheets>
     <sheet name="Entry List" sheetId="1" r:id="rId1"/>
@@ -40,6 +40,7 @@
     <sheet name="MarkerTrait data" sheetId="23" r:id="rId25"/>
     <sheet name="Marker info" sheetId="30" r:id="rId26"/>
     <sheet name="African stem rust" sheetId="36" r:id="rId27"/>
+    <sheet name="Sheet1" sheetId="37" r:id="rId28"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -60,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4582" uniqueCount="750">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4583" uniqueCount="751">
   <si>
     <t>Entry</t>
   </si>
@@ -3412,6 +3413,9 @@
   </si>
   <si>
     <t>Previous crop: Flax. Soil type: Williams-Bowbells loam. Rainfall: 7.8 inches (4/26 - 8/16)</t>
+  </si>
+  <si>
+    <t>Hannah testing</t>
   </si>
 </sst>
 </file>
@@ -5839,6 +5843,9 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -5872,14 +5879,11 @@
     <xf numFmtId="0" fontId="68" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="126">
@@ -14240,14 +14244,14 @@
       <c r="A3" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="339" t="s">
+      <c r="B3" s="340" t="s">
         <v>69</v>
       </c>
-      <c r="C3" s="339"/>
-      <c r="D3" s="339" t="s">
+      <c r="C3" s="340"/>
+      <c r="D3" s="340" t="s">
         <v>70</v>
       </c>
-      <c r="E3" s="339"/>
+      <c r="E3" s="340"/>
       <c r="F3" s="31" t="s">
         <v>71</v>
       </c>
@@ -14265,14 +14269,14 @@
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="2"/>
-      <c r="B4" s="339" t="s">
+      <c r="B4" s="340" t="s">
         <v>75</v>
       </c>
-      <c r="C4" s="339"/>
-      <c r="D4" s="339" t="s">
+      <c r="C4" s="340"/>
+      <c r="D4" s="340" t="s">
         <v>76</v>
       </c>
-      <c r="E4" s="339"/>
+      <c r="E4" s="340"/>
       <c r="F4" s="31" t="s">
         <v>77</v>
       </c>
@@ -17284,43 +17288,43 @@
     <row r="4" spans="1:15" ht="15" customHeight="1">
       <c r="A4" s="27"/>
       <c r="B4" s="27"/>
-      <c r="C4" s="340" t="s">
+      <c r="C4" s="341" t="s">
         <v>237</v>
       </c>
-      <c r="D4" s="340" t="s">
+      <c r="D4" s="341" t="s">
         <v>362</v>
       </c>
-      <c r="E4" s="344" t="s">
+      <c r="E4" s="345" t="s">
         <v>351</v>
       </c>
-      <c r="F4" s="344" t="s">
+      <c r="F4" s="345" t="s">
         <v>352</v>
       </c>
-      <c r="G4" s="344" t="s">
+      <c r="G4" s="345" t="s">
         <v>353</v>
       </c>
-      <c r="H4" s="344" t="s">
+      <c r="H4" s="345" t="s">
         <v>354</v>
       </c>
-      <c r="I4" s="344" t="s">
+      <c r="I4" s="345" t="s">
         <v>355</v>
       </c>
-      <c r="J4" s="344" t="s">
+      <c r="J4" s="345" t="s">
         <v>356</v>
       </c>
-      <c r="K4" s="344" t="s">
+      <c r="K4" s="345" t="s">
         <v>357</v>
       </c>
-      <c r="L4" s="344" t="s">
+      <c r="L4" s="345" t="s">
         <v>358</v>
       </c>
-      <c r="M4" s="344" t="s">
+      <c r="M4" s="345" t="s">
         <v>359</v>
       </c>
-      <c r="N4" s="344" t="s">
+      <c r="N4" s="345" t="s">
         <v>360</v>
       </c>
-      <c r="O4" s="342" t="s">
+      <c r="O4" s="343" t="s">
         <v>361</v>
       </c>
     </row>
@@ -17331,19 +17335,19 @@
       <c r="B5" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="341"/>
-      <c r="D5" s="341"/>
-      <c r="E5" s="345"/>
-      <c r="F5" s="345"/>
-      <c r="G5" s="345"/>
-      <c r="H5" s="345"/>
-      <c r="I5" s="345"/>
-      <c r="J5" s="345"/>
-      <c r="K5" s="345"/>
-      <c r="L5" s="345"/>
-      <c r="M5" s="345"/>
-      <c r="N5" s="345"/>
-      <c r="O5" s="343"/>
+      <c r="C5" s="342"/>
+      <c r="D5" s="342"/>
+      <c r="E5" s="346"/>
+      <c r="F5" s="346"/>
+      <c r="G5" s="346"/>
+      <c r="H5" s="346"/>
+      <c r="I5" s="346"/>
+      <c r="J5" s="346"/>
+      <c r="K5" s="346"/>
+      <c r="L5" s="346"/>
+      <c r="M5" s="346"/>
+      <c r="N5" s="346"/>
+      <c r="O5" s="344"/>
     </row>
     <row r="6" spans="1:15" ht="12.75" customHeight="1" thickTop="1">
       <c r="A6" s="13">
@@ -18880,19 +18884,19 @@
     <row r="3" spans="1:9">
       <c r="A3" s="38"/>
       <c r="B3" s="38"/>
-      <c r="C3" s="338" t="s">
+      <c r="C3" s="339" t="s">
         <v>94</v>
       </c>
-      <c r="D3" s="338"/>
+      <c r="D3" s="339"/>
       <c r="E3" s="9"/>
       <c r="F3" s="60" t="s">
         <v>95</v>
       </c>
       <c r="G3" s="9"/>
-      <c r="H3" s="338" t="s">
+      <c r="H3" s="339" t="s">
         <v>96</v>
       </c>
-      <c r="I3" s="338"/>
+      <c r="I3" s="339"/>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="38"/>
@@ -21673,17 +21677,17 @@
       <c r="N18" s="15"/>
     </row>
     <row r="19" spans="1:14" ht="23.25" customHeight="1">
-      <c r="A19" s="346" t="s">
+      <c r="A19" s="347" t="s">
         <v>123</v>
       </c>
-      <c r="B19" s="346"/>
-      <c r="C19" s="346"/>
-      <c r="D19" s="346"/>
-      <c r="E19" s="346"/>
-      <c r="F19" s="346"/>
-      <c r="G19" s="346"/>
-      <c r="H19" s="346"/>
-      <c r="I19" s="346"/>
+      <c r="B19" s="347"/>
+      <c r="C19" s="347"/>
+      <c r="D19" s="347"/>
+      <c r="E19" s="347"/>
+      <c r="F19" s="347"/>
+      <c r="G19" s="347"/>
+      <c r="H19" s="347"/>
+      <c r="I19" s="347"/>
       <c r="J19" s="69"/>
       <c r="K19" s="70"/>
       <c r="L19" s="71"/>
@@ -21853,17 +21857,17 @@
       <c r="I31" s="164"/>
     </row>
     <row r="32" spans="1:14" ht="23.25" customHeight="1">
-      <c r="A32" s="347" t="s">
+      <c r="A32" s="348" t="s">
         <v>408</v>
       </c>
-      <c r="B32" s="347"/>
-      <c r="C32" s="347"/>
-      <c r="D32" s="347"/>
-      <c r="E32" s="347"/>
-      <c r="F32" s="347"/>
-      <c r="G32" s="347"/>
-      <c r="H32" s="347"/>
-      <c r="I32" s="347"/>
+      <c r="B32" s="348"/>
+      <c r="C32" s="348"/>
+      <c r="D32" s="348"/>
+      <c r="E32" s="348"/>
+      <c r="F32" s="348"/>
+      <c r="G32" s="348"/>
+      <c r="H32" s="348"/>
+      <c r="I32" s="348"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -23014,25 +23018,25 @@
         <v>81</v>
       </c>
       <c r="B41" s="3"/>
-      <c r="C41" s="349">
+      <c r="C41" s="338">
         <v>23.125</v>
       </c>
-      <c r="D41" s="349">
+      <c r="D41" s="338">
         <v>90.555555555555557</v>
       </c>
-      <c r="E41" s="349">
+      <c r="E41" s="338">
         <v>19.029166666666669</v>
       </c>
-      <c r="F41" s="349">
+      <c r="F41" s="338">
         <v>18.226388888888888</v>
       </c>
-      <c r="G41" s="349">
+      <c r="G41" s="338">
         <v>11.101388888888888</v>
       </c>
-      <c r="H41" s="349">
+      <c r="H41" s="338">
         <v>17.972222222222221</v>
       </c>
-      <c r="I41" s="349">
+      <c r="I41" s="338">
         <v>4.1638888888888879</v>
       </c>
     </row>
@@ -24001,16 +24005,16 @@
         <v>81</v>
       </c>
       <c r="B41" s="3"/>
-      <c r="C41" s="349">
+      <c r="C41" s="338">
         <v>37.666666666666664</v>
       </c>
-      <c r="D41" s="349">
+      <c r="D41" s="338">
         <v>10.666197183098591</v>
       </c>
-      <c r="E41" s="349">
+      <c r="E41" s="338">
         <v>24.652777777777779</v>
       </c>
-      <c r="F41" s="349">
+      <c r="F41" s="338">
         <v>17.441666666666663</v>
       </c>
     </row>
@@ -27846,7 +27850,7 @@
     </row>
     <row r="41" spans="1:26" ht="141" customHeight="1">
       <c r="A41" s="13"/>
-      <c r="B41" s="348" t="s">
+      <c r="B41" s="349" t="s">
         <v>64</v>
       </c>
       <c r="C41" s="134" t="s">
@@ -27924,7 +27928,7 @@
     </row>
     <row r="42" spans="1:26" ht="141" customHeight="1">
       <c r="A42" s="13"/>
-      <c r="B42" s="348"/>
+      <c r="B42" s="349"/>
       <c r="C42" s="134" t="s">
         <v>141</v>
       </c>
@@ -35798,16 +35802,16 @@
       </c>
     </row>
     <row r="67" spans="1:53" ht="38.25" customHeight="1">
-      <c r="A67" s="351" t="s">
+      <c r="A67" s="350" t="s">
         <v>686</v>
       </c>
-      <c r="B67" s="351"/>
-      <c r="C67" s="351"/>
-      <c r="D67" s="351"/>
-      <c r="E67" s="351"/>
-      <c r="F67" s="351"/>
-      <c r="G67" s="351"/>
-      <c r="H67" s="351"/>
+      <c r="B67" s="350"/>
+      <c r="C67" s="350"/>
+      <c r="D67" s="350"/>
+      <c r="E67" s="350"/>
+      <c r="F67" s="350"/>
+      <c r="G67" s="350"/>
+      <c r="H67" s="350"/>
       <c r="I67" s="38"/>
       <c r="J67" s="38"/>
       <c r="K67" s="38"/>
@@ -35912,16 +35916,16 @@
       <c r="BA68" s="38"/>
     </row>
     <row r="69" spans="1:53" ht="25.5" customHeight="1">
-      <c r="A69" s="350" t="s">
+      <c r="A69" s="351" t="s">
         <v>688</v>
       </c>
-      <c r="B69" s="350"/>
-      <c r="C69" s="350"/>
-      <c r="D69" s="350"/>
-      <c r="E69" s="350"/>
-      <c r="F69" s="350"/>
-      <c r="G69" s="350"/>
-      <c r="H69" s="350"/>
+      <c r="B69" s="351"/>
+      <c r="C69" s="351"/>
+      <c r="D69" s="351"/>
+      <c r="E69" s="351"/>
+      <c r="F69" s="351"/>
+      <c r="G69" s="351"/>
+      <c r="H69" s="351"/>
       <c r="I69" s="38"/>
       <c r="J69" s="38"/>
       <c r="K69" s="38"/>
@@ -35969,16 +35973,16 @@
       <c r="BA69" s="38"/>
     </row>
     <row r="70" spans="1:53" ht="25.5" customHeight="1">
-      <c r="A70" s="350" t="s">
+      <c r="A70" s="351" t="s">
         <v>689</v>
       </c>
-      <c r="B70" s="350"/>
-      <c r="C70" s="350"/>
-      <c r="D70" s="350"/>
-      <c r="E70" s="350"/>
-      <c r="F70" s="350"/>
-      <c r="G70" s="350"/>
-      <c r="H70" s="350"/>
+      <c r="B70" s="351"/>
+      <c r="C70" s="351"/>
+      <c r="D70" s="351"/>
+      <c r="E70" s="351"/>
+      <c r="F70" s="351"/>
+      <c r="G70" s="351"/>
+      <c r="H70" s="351"/>
       <c r="I70" s="38"/>
       <c r="J70" s="38"/>
       <c r="K70" s="38"/>
@@ -36231,6 +36235,21 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C79DBE69-9EA5-4910-8382-7DB3FFCE54DB}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" t="s">
+        <v>750</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E61D2DC-DC32-47AE-9144-9665F814590A}">
   <dimension ref="A1:G47"/>

</xml_diff>